<commit_message>
Update report Register TestCase
</commit_message>
<xml_diff>
--- a/TestCases/Register_TestCase.xlsx
+++ b/TestCases/Register_TestCase.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DoAnNganh\SpringMediCareWeb-Selenium-Testing\TestCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBDCC797-BD68-41AE-8BA5-C232F79EDAE2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B75FE8B-1885-45F1-A7A9-8A48D5CA5FF4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name=" Register" sheetId="4" r:id="rId1"/>
+    <sheet name="Register" sheetId="4" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="ACTION">#REF!</definedName>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="141">
   <si>
     <t>TEST CASE</t>
   </si>
@@ -315,6 +315,9 @@
     <t>Hệ thống vẫn cho phép đăng ký với số điện thoại 11 chữ số và chuyển đến trang đăng nhập, không hiển thị thông báo số điện thoại không hợp lệ.</t>
   </si>
   <si>
+    <t>TCRegisterRetest11</t>
+  </si>
+  <si>
     <t>TC-REGISTER-012</t>
   </si>
   <si>
@@ -359,6 +362,9 @@
     <t>Hệ thống vẫn cho phép đăng ký với mật khẩu chỉ có 6 ký tự và chuyển đến trang đăng nhập, không hiển thị thông báo mật khẩu không hợp lệ.</t>
   </si>
   <si>
+    <t>TCRegisterRetest13</t>
+  </si>
+  <si>
     <t>TC-REGISTER-014</t>
   </si>
   <si>
@@ -379,6 +385,9 @@
   </si>
   <si>
     <t>Hệ thống vẫn cho phép đăng ký với mật khẩu không có ký tự hoa và chuyển đến trang đăng nhập, không hiển thị thông báo mật khẩu không hợp lệ.</t>
+  </si>
+  <si>
+    <t>TCRegisterRetest14</t>
   </si>
   <si>
     <t>TC-REGISTER-015</t>
@@ -403,6 +412,9 @@
     <t>Hệ thống vẫn cho phép đăng ký với mật khẩu không có chữ thường và chuyển đến trang đăng nhập, không hiển thị thông báo mật khẩu không hợp lệ.</t>
   </si>
   <si>
+    <t>TCRegisterRetest15</t>
+  </si>
+  <si>
     <t>TC-REGISTER-016</t>
   </si>
   <si>
@@ -423,6 +435,9 @@
   </si>
   <si>
     <t>Hệ thống vẫn cho phép đăng ký với mật khẩu không có chữ số và chuyển đến trang đăng nhập, không hiển thị thông báo mật khẩu không hợp lệ.</t>
+  </si>
+  <si>
+    <t>TCRegisterRetest16</t>
   </si>
   <si>
     <t>TC-REGISTER-017</t>
@@ -447,6 +462,9 @@
     <t>Hệ thống vẫn cho phép đăng ký với mật khẩu không có ký tự đặc biệt và chuyển đến trang đăng nhập, không hiển thị thông báo mật khẩu không hợp lệ.</t>
   </si>
   <si>
+    <t>TCRegisterRetest17</t>
+  </si>
+  <si>
     <t xml:space="preserve">4. Kiểm tra dữ liệu đã tồn tại     </t>
   </si>
   <si>
@@ -469,7 +487,10 @@
     <t>TCRegister18_1, TCRegister18_2</t>
   </si>
   <si>
-    <t>Hệ thống không tạo tài khoản và hiển thị thông báo vui lòng kiểm tra lại thông tin.</t>
+    <t>Hệ thống chưa hiển thị thông báo cụ thể khi người dùng đăng ký bằng tên đăng nhập đã tồn tại.</t>
+  </si>
+  <si>
+    <t>TCRegisterRetest18</t>
   </si>
   <si>
     <t>TC-REGISTER-019</t>
@@ -492,6 +513,9 @@
   <si>
     <t>Hệ thống vẫn cho phép đăng ký tài khoản với email đã tồn tại</t>
   </si>
+  <si>
+    <t>TCRegisterRetest19</t>
+  </si>
 </sst>
 </file>
 
@@ -500,7 +524,7 @@
   <numFmts count="1">
     <numFmt numFmtId="166" formatCode="d\-m"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -548,6 +572,12 @@
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Tahoma"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
     </font>
     <font>
       <sz val="11"/>
@@ -717,7 +747,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
@@ -761,7 +791,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1022,16 +1055,16 @@
     <col min="9" max="9" width="15.44140625" customWidth="1"/>
     <col min="10" max="10" width="21.33203125" customWidth="1"/>
     <col min="11" max="12" width="19.88671875" customWidth="1"/>
-    <col min="13" max="13" width="21.109375" customWidth="1"/>
+    <col min="13" max="13" width="22.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -1058,9 +1091,9 @@
     </row>
     <row r="2" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -1089,11 +1122,11 @@
       <c r="A3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="22"/>
-      <c r="D3" s="24"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="25"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -1122,11 +1155,11 @@
       <c r="A4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="22"/>
-      <c r="D4" s="24"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="25"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -1155,11 +1188,11 @@
       <c r="A5" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B5" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="22"/>
-      <c r="D5" s="24"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="25"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -1288,39 +1321,39 @@
       <c r="AA8" s="3"/>
     </row>
     <row r="9" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A9" s="31" t="s">
+      <c r="A9" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="31" t="s">
+      <c r="C9" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="33" t="s">
+      <c r="D9" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="31" t="s">
+      <c r="E9" s="29"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="34" t="s">
+      <c r="H9" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="I9" s="34" t="s">
+      <c r="I9" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="J9" s="34" t="s">
+      <c r="J9" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="K9" s="34" t="s">
+      <c r="K9" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="L9" s="34" t="s">
+      <c r="L9" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="M9" s="34" t="s">
+      <c r="M9" s="35" t="s">
         <v>20</v>
       </c>
       <c r="N9" s="3"/>
@@ -1339,19 +1372,19 @@
       <c r="AA9" s="3"/>
     </row>
     <row r="10" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A10" s="23"/>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="25"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="23"/>
-      <c r="J10" s="23"/>
-      <c r="K10" s="23"/>
-      <c r="L10" s="23"/>
-      <c r="M10" s="23"/>
+      <c r="A10" s="24"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="24"/>
+      <c r="J10" s="24"/>
+      <c r="K10" s="24"/>
+      <c r="L10" s="24"/>
+      <c r="M10" s="24"/>
       <c r="N10" s="3"/>
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
@@ -1373,14 +1406,14 @@
       <c r="C11" s="11"/>
       <c r="D11" s="11"/>
       <c r="E11" s="11"/>
-      <c r="F11" s="35"/>
-      <c r="G11" s="22"/>
-      <c r="H11" s="22"/>
-      <c r="I11" s="22"/>
-      <c r="J11" s="22"/>
-      <c r="K11" s="22"/>
-      <c r="L11" s="22"/>
-      <c r="M11" s="22"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
+      <c r="J11" s="23"/>
+      <c r="K11" s="23"/>
+      <c r="L11" s="23"/>
+      <c r="M11" s="23"/>
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
@@ -1397,21 +1430,21 @@
       <c r="AA11" s="3"/>
     </row>
     <row r="12" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A12" s="36" t="s">
+      <c r="A12" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="22"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="22"/>
-      <c r="I12" s="22"/>
-      <c r="J12" s="22"/>
-      <c r="K12" s="22"/>
-      <c r="L12" s="22"/>
-      <c r="M12" s="24"/>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="23"/>
+      <c r="J12" s="23"/>
+      <c r="K12" s="23"/>
+      <c r="L12" s="23"/>
+      <c r="M12" s="25"/>
       <c r="N12" s="3"/>
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
@@ -1437,11 +1470,11 @@
       <c r="C13" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="37" t="s">
+      <c r="D13" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
       <c r="G13" s="17" t="s">
         <v>30</v>
       </c>
@@ -1473,21 +1506,21 @@
       <c r="AA13" s="3"/>
     </row>
     <row r="14" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A14" s="36" t="s">
+      <c r="A14" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="22"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="22"/>
-      <c r="H14" s="22"/>
-      <c r="I14" s="22"/>
-      <c r="J14" s="22"/>
-      <c r="K14" s="22"/>
-      <c r="L14" s="22"/>
-      <c r="M14" s="24"/>
+      <c r="B14" s="23"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
+      <c r="H14" s="23"/>
+      <c r="I14" s="23"/>
+      <c r="J14" s="23"/>
+      <c r="K14" s="23"/>
+      <c r="L14" s="23"/>
+      <c r="M14" s="25"/>
       <c r="N14" s="3"/>
       <c r="O14" s="3"/>
       <c r="P14" s="3"/>
@@ -1513,11 +1546,11 @@
       <c r="C15" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="D15" s="37" t="s">
+      <c r="D15" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="23"/>
       <c r="G15" s="17" t="s">
         <v>36</v>
       </c>
@@ -1558,11 +1591,11 @@
       <c r="C16" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="D16" s="37" t="s">
+      <c r="D16" s="38" t="s">
         <v>41</v>
       </c>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
       <c r="G16" s="17" t="s">
         <v>42</v>
       </c>
@@ -1603,11 +1636,11 @@
       <c r="C17" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="D17" s="37" t="s">
+      <c r="D17" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
       <c r="G17" s="17" t="s">
         <v>47</v>
       </c>
@@ -1648,11 +1681,11 @@
       <c r="C18" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="D18" s="37" t="s">
+      <c r="D18" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="23"/>
       <c r="G18" s="17" t="s">
         <v>52</v>
       </c>
@@ -1693,11 +1726,11 @@
       <c r="C19" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="D19" s="37" t="s">
+      <c r="D19" s="38" t="s">
         <v>56</v>
       </c>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="23"/>
       <c r="G19" s="17" t="s">
         <v>57</v>
       </c>
@@ -1738,11 +1771,11 @@
       <c r="C20" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="D20" s="37" t="s">
+      <c r="D20" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="23"/>
       <c r="G20" s="17" t="s">
         <v>61</v>
       </c>
@@ -1783,11 +1816,11 @@
       <c r="C21" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="D21" s="37" t="s">
+      <c r="D21" s="38" t="s">
         <v>64</v>
       </c>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
+      <c r="E21" s="23"/>
+      <c r="F21" s="23"/>
       <c r="G21" s="17" t="s">
         <v>65</v>
       </c>
@@ -1828,11 +1861,11 @@
       <c r="C22" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="D22" s="37" t="s">
+      <c r="D22" s="38" t="s">
         <v>69</v>
       </c>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="23"/>
       <c r="G22" s="17" t="s">
         <v>70</v>
       </c>
@@ -1864,21 +1897,21 @@
       <c r="AA22" s="3"/>
     </row>
     <row r="23" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A23" s="36" t="s">
+      <c r="A23" s="37" t="s">
         <v>71</v>
       </c>
-      <c r="B23" s="22"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="22"/>
-      <c r="H23" s="22"/>
-      <c r="I23" s="22"/>
-      <c r="J23" s="22"/>
-      <c r="K23" s="22"/>
-      <c r="L23" s="22"/>
-      <c r="M23" s="24"/>
+      <c r="B23" s="23"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="23"/>
+      <c r="G23" s="23"/>
+      <c r="H23" s="23"/>
+      <c r="I23" s="23"/>
+      <c r="J23" s="23"/>
+      <c r="K23" s="23"/>
+      <c r="L23" s="23"/>
+      <c r="M23" s="25"/>
       <c r="N23" s="3"/>
       <c r="O23" s="3"/>
       <c r="P23" s="3"/>
@@ -1904,11 +1937,11 @@
       <c r="C24" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="D24" s="37" t="s">
+      <c r="D24" s="38" t="s">
         <v>75</v>
       </c>
-      <c r="E24" s="22"/>
-      <c r="F24" s="22"/>
+      <c r="E24" s="23"/>
+      <c r="F24" s="23"/>
       <c r="G24" s="17" t="s">
         <v>76</v>
       </c>
@@ -1949,11 +1982,11 @@
       <c r="C25" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="D25" s="37" t="s">
+      <c r="D25" s="38" t="s">
         <v>81</v>
       </c>
-      <c r="E25" s="22"/>
-      <c r="F25" s="22"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="23"/>
       <c r="G25" s="17" t="s">
         <v>82</v>
       </c>
@@ -1966,9 +1999,15 @@
       <c r="J25" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="K25" s="19"/>
-      <c r="L25" s="19"/>
-      <c r="M25" s="20"/>
+      <c r="K25" s="18">
+        <v>46219</v>
+      </c>
+      <c r="L25" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="M25" s="21" t="s">
+        <v>84</v>
+      </c>
       <c r="N25" s="3"/>
       <c r="O25" s="3"/>
       <c r="P25" s="3"/>
@@ -1986,21 +2025,21 @@
     </row>
     <row r="26" spans="1:27" ht="84.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>86</v>
-      </c>
-      <c r="D26" s="37" t="s">
         <v>87</v>
       </c>
-      <c r="E26" s="22"/>
-      <c r="F26" s="22"/>
+      <c r="D26" s="38" t="s">
+        <v>88</v>
+      </c>
+      <c r="E26" s="23"/>
+      <c r="F26" s="23"/>
       <c r="G26" s="17" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H26" s="18">
         <v>46218</v>
@@ -2009,7 +2048,7 @@
         <v>2</v>
       </c>
       <c r="J26" s="16" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K26" s="19"/>
       <c r="L26" s="19"/>
@@ -2031,21 +2070,21 @@
     </row>
     <row r="27" spans="1:27" ht="84.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>92</v>
-      </c>
-      <c r="D27" s="37" t="s">
         <v>93</v>
       </c>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
+      <c r="D27" s="38" t="s">
+        <v>94</v>
+      </c>
+      <c r="E27" s="23"/>
+      <c r="F27" s="23"/>
       <c r="G27" s="17" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H27" s="18">
         <v>46218</v>
@@ -2054,11 +2093,17 @@
         <v>4</v>
       </c>
       <c r="J27" s="16" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
-      <c r="K27" s="19"/>
-      <c r="L27" s="19"/>
-      <c r="M27" s="20"/>
+      <c r="K27" s="18">
+        <v>46219</v>
+      </c>
+      <c r="L27" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="M27" s="21" t="s">
+        <v>97</v>
+      </c>
       <c r="N27" s="3"/>
       <c r="O27" s="3"/>
       <c r="P27" s="3"/>
@@ -2076,21 +2121,21 @@
     </row>
     <row r="28" spans="1:27" ht="106.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
-      <c r="D28" s="37" t="s">
-        <v>99</v>
+      <c r="D28" s="38" t="s">
+        <v>101</v>
       </c>
-      <c r="E28" s="22"/>
-      <c r="F28" s="22"/>
+      <c r="E28" s="23"/>
+      <c r="F28" s="23"/>
       <c r="G28" s="17" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H28" s="18">
         <v>46218</v>
@@ -2099,11 +2144,17 @@
         <v>4</v>
       </c>
       <c r="J28" s="16" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
-      <c r="K28" s="19"/>
-      <c r="L28" s="19"/>
-      <c r="M28" s="20"/>
+      <c r="K28" s="18">
+        <v>46219</v>
+      </c>
+      <c r="L28" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="M28" s="21" t="s">
+        <v>104</v>
+      </c>
       <c r="N28" s="3"/>
       <c r="O28" s="3"/>
       <c r="P28" s="3"/>
@@ -2121,21 +2172,21 @@
     </row>
     <row r="29" spans="1:27" ht="108.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
-      <c r="D29" s="37" t="s">
-        <v>105</v>
+      <c r="D29" s="38" t="s">
+        <v>108</v>
       </c>
-      <c r="E29" s="22"/>
-      <c r="F29" s="22"/>
+      <c r="E29" s="23"/>
+      <c r="F29" s="23"/>
       <c r="G29" s="17" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H29" s="18">
         <v>46218</v>
@@ -2144,11 +2195,17 @@
         <v>4</v>
       </c>
       <c r="J29" s="16" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
-      <c r="K29" s="19"/>
-      <c r="L29" s="19"/>
-      <c r="M29" s="20"/>
+      <c r="K29" s="18">
+        <v>46219</v>
+      </c>
+      <c r="L29" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="M29" s="21" t="s">
+        <v>111</v>
+      </c>
       <c r="N29" s="3"/>
       <c r="O29" s="3"/>
       <c r="P29" s="3"/>
@@ -2166,21 +2223,21 @@
     </row>
     <row r="30" spans="1:27" ht="108.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
-      <c r="D30" s="37" t="s">
-        <v>111</v>
+      <c r="D30" s="38" t="s">
+        <v>115</v>
       </c>
-      <c r="E30" s="22"/>
-      <c r="F30" s="22"/>
+      <c r="E30" s="23"/>
+      <c r="F30" s="23"/>
       <c r="G30" s="17" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="H30" s="18">
         <v>46218</v>
@@ -2189,11 +2246,17 @@
         <v>4</v>
       </c>
       <c r="J30" s="16" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
-      <c r="K30" s="19"/>
-      <c r="L30" s="19"/>
-      <c r="M30" s="20"/>
+      <c r="K30" s="18">
+        <v>46219</v>
+      </c>
+      <c r="L30" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="M30" s="21" t="s">
+        <v>118</v>
+      </c>
       <c r="N30" s="3"/>
       <c r="O30" s="3"/>
       <c r="P30" s="3"/>
@@ -2211,21 +2274,21 @@
     </row>
     <row r="31" spans="1:27" ht="108.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
-      <c r="D31" s="37" t="s">
-        <v>117</v>
+      <c r="D31" s="38" t="s">
+        <v>122</v>
       </c>
-      <c r="E31" s="22"/>
-      <c r="F31" s="22"/>
+      <c r="E31" s="23"/>
+      <c r="F31" s="23"/>
       <c r="G31" s="17" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="H31" s="18">
         <v>46218</v>
@@ -2234,11 +2297,17 @@
         <v>4</v>
       </c>
       <c r="J31" s="16" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
-      <c r="K31" s="19"/>
-      <c r="L31" s="19"/>
-      <c r="M31" s="20"/>
+      <c r="K31" s="18">
+        <v>46219</v>
+      </c>
+      <c r="L31" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="M31" s="21" t="s">
+        <v>125</v>
+      </c>
       <c r="N31" s="3"/>
       <c r="O31" s="3"/>
       <c r="P31" s="3"/>
@@ -2255,21 +2324,21 @@
       <c r="AA31" s="3"/>
     </row>
     <row r="32" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A32" s="36" t="s">
-        <v>120</v>
+      <c r="A32" s="37" t="s">
+        <v>126</v>
       </c>
-      <c r="B32" s="22"/>
-      <c r="C32" s="22"/>
-      <c r="D32" s="22"/>
-      <c r="E32" s="22"/>
-      <c r="F32" s="22"/>
-      <c r="G32" s="22"/>
-      <c r="H32" s="22"/>
-      <c r="I32" s="22"/>
-      <c r="J32" s="22"/>
-      <c r="K32" s="22"/>
-      <c r="L32" s="22"/>
-      <c r="M32" s="24"/>
+      <c r="B32" s="23"/>
+      <c r="C32" s="23"/>
+      <c r="D32" s="23"/>
+      <c r="E32" s="23"/>
+      <c r="F32" s="23"/>
+      <c r="G32" s="23"/>
+      <c r="H32" s="23"/>
+      <c r="I32" s="23"/>
+      <c r="J32" s="23"/>
+      <c r="K32" s="23"/>
+      <c r="L32" s="23"/>
+      <c r="M32" s="25"/>
       <c r="N32" s="3"/>
       <c r="O32" s="3"/>
       <c r="P32" s="3"/>
@@ -2287,34 +2356,40 @@
     </row>
     <row r="33" spans="1:27" ht="69" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
-      <c r="D33" s="37" t="s">
-        <v>124</v>
+      <c r="D33" s="38" t="s">
+        <v>130</v>
       </c>
-      <c r="E33" s="22"/>
-      <c r="F33" s="22"/>
+      <c r="E33" s="23"/>
+      <c r="F33" s="23"/>
       <c r="G33" s="17" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="H33" s="18">
         <v>46218</v>
       </c>
       <c r="I33" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="J33" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="K33" s="18">
+        <v>46219</v>
+      </c>
+      <c r="L33" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="J33" s="16" t="s">
-        <v>126</v>
+      <c r="M33" s="21" t="s">
+        <v>133</v>
       </c>
-      <c r="K33" s="19"/>
-      <c r="L33" s="19"/>
-      <c r="M33" s="20"/>
       <c r="N33" s="3"/>
       <c r="O33" s="3"/>
       <c r="P33" s="3"/>
@@ -2330,23 +2405,23 @@
       <c r="Z33" s="3"/>
       <c r="AA33" s="3"/>
     </row>
-    <row r="34" spans="1:27" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:27" ht="75.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="14" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
-      <c r="D34" s="37" t="s">
-        <v>130</v>
+      <c r="D34" s="38" t="s">
+        <v>137</v>
       </c>
-      <c r="E34" s="22"/>
-      <c r="F34" s="22"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="23"/>
       <c r="G34" s="17" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="H34" s="18">
         <v>46218</v>
@@ -2355,11 +2430,17 @@
         <v>4</v>
       </c>
       <c r="J34" s="16" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
-      <c r="K34" s="19"/>
-      <c r="L34" s="19"/>
-      <c r="M34" s="20"/>
+      <c r="K34" s="18">
+        <v>46219</v>
+      </c>
+      <c r="L34" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="M34" s="21" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="35" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A35" s="3"/>
@@ -30666,33 +30747,33 @@
       <c r="AA1010" s="3"/>
     </row>
     <row r="1011" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A1011" s="21"/>
-      <c r="B1011" s="21"/>
-      <c r="C1011" s="21"/>
-      <c r="D1011" s="21"/>
-      <c r="E1011" s="21"/>
-      <c r="F1011" s="21"/>
-      <c r="G1011" s="21"/>
-      <c r="H1011" s="21"/>
-      <c r="I1011" s="21"/>
-      <c r="J1011" s="21"/>
-      <c r="K1011" s="21"/>
-      <c r="L1011" s="21"/>
-      <c r="M1011" s="21"/>
-      <c r="N1011" s="21"/>
-      <c r="O1011" s="21"/>
-      <c r="P1011" s="21"/>
-      <c r="Q1011" s="21"/>
-      <c r="R1011" s="21"/>
-      <c r="S1011" s="21"/>
-      <c r="T1011" s="21"/>
-      <c r="U1011" s="21"/>
-      <c r="V1011" s="21"/>
-      <c r="W1011" s="21"/>
-      <c r="X1011" s="21"/>
-      <c r="Y1011" s="21"/>
-      <c r="Z1011" s="21"/>
-      <c r="AA1011" s="21"/>
+      <c r="A1011" s="22"/>
+      <c r="B1011" s="22"/>
+      <c r="C1011" s="22"/>
+      <c r="D1011" s="22"/>
+      <c r="E1011" s="22"/>
+      <c r="F1011" s="22"/>
+      <c r="G1011" s="22"/>
+      <c r="H1011" s="22"/>
+      <c r="I1011" s="22"/>
+      <c r="J1011" s="22"/>
+      <c r="K1011" s="22"/>
+      <c r="L1011" s="22"/>
+      <c r="M1011" s="22"/>
+      <c r="N1011" s="22"/>
+      <c r="O1011" s="22"/>
+      <c r="P1011" s="22"/>
+      <c r="Q1011" s="22"/>
+      <c r="R1011" s="22"/>
+      <c r="S1011" s="22"/>
+      <c r="T1011" s="22"/>
+      <c r="U1011" s="22"/>
+      <c r="V1011" s="22"/>
+      <c r="W1011" s="22"/>
+      <c r="X1011" s="22"/>
+      <c r="Y1011" s="22"/>
+      <c r="Z1011" s="22"/>
+      <c r="AA1011" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="39">
@@ -30748,14 +30829,22 @@
     <hyperlink ref="G22" r:id="rId9" xr:uid="{00000000-0004-0000-0300-000008000000}"/>
     <hyperlink ref="G24" r:id="rId10" xr:uid="{00000000-0004-0000-0300-000009000000}"/>
     <hyperlink ref="G25" r:id="rId11" xr:uid="{00000000-0004-0000-0300-00000A000000}"/>
-    <hyperlink ref="G26" r:id="rId12" xr:uid="{00000000-0004-0000-0300-00000B000000}"/>
-    <hyperlink ref="G27" r:id="rId13" xr:uid="{00000000-0004-0000-0300-00000C000000}"/>
-    <hyperlink ref="G28" r:id="rId14" xr:uid="{00000000-0004-0000-0300-00000D000000}"/>
-    <hyperlink ref="G29" r:id="rId15" xr:uid="{00000000-0004-0000-0300-00000E000000}"/>
-    <hyperlink ref="G30" r:id="rId16" xr:uid="{00000000-0004-0000-0300-00000F000000}"/>
-    <hyperlink ref="G31" r:id="rId17" xr:uid="{00000000-0004-0000-0300-000010000000}"/>
-    <hyperlink ref="G33" r:id="rId18" xr:uid="{00000000-0004-0000-0300-000011000000}"/>
-    <hyperlink ref="G34" r:id="rId19" xr:uid="{00000000-0004-0000-0300-000012000000}"/>
+    <hyperlink ref="M25" r:id="rId12" xr:uid="{00000000-0004-0000-0300-00000B000000}"/>
+    <hyperlink ref="G26" r:id="rId13" xr:uid="{00000000-0004-0000-0300-00000C000000}"/>
+    <hyperlink ref="G27" r:id="rId14" xr:uid="{00000000-0004-0000-0300-00000D000000}"/>
+    <hyperlink ref="M27" r:id="rId15" xr:uid="{00000000-0004-0000-0300-00000E000000}"/>
+    <hyperlink ref="G28" r:id="rId16" xr:uid="{00000000-0004-0000-0300-00000F000000}"/>
+    <hyperlink ref="M28" r:id="rId17" xr:uid="{00000000-0004-0000-0300-000010000000}"/>
+    <hyperlink ref="G29" r:id="rId18" xr:uid="{00000000-0004-0000-0300-000011000000}"/>
+    <hyperlink ref="M29" r:id="rId19" xr:uid="{00000000-0004-0000-0300-000012000000}"/>
+    <hyperlink ref="G30" r:id="rId20" xr:uid="{00000000-0004-0000-0300-000013000000}"/>
+    <hyperlink ref="M30" r:id="rId21" xr:uid="{00000000-0004-0000-0300-000014000000}"/>
+    <hyperlink ref="G31" r:id="rId22" xr:uid="{00000000-0004-0000-0300-000015000000}"/>
+    <hyperlink ref="M31" r:id="rId23" xr:uid="{00000000-0004-0000-0300-000016000000}"/>
+    <hyperlink ref="G33" r:id="rId24" xr:uid="{00000000-0004-0000-0300-000017000000}"/>
+    <hyperlink ref="M33" r:id="rId25" xr:uid="{00000000-0004-0000-0300-000018000000}"/>
+    <hyperlink ref="G34" r:id="rId26" xr:uid="{00000000-0004-0000-0300-000019000000}"/>
+    <hyperlink ref="M34" r:id="rId27" xr:uid="{00000000-0004-0000-0300-00001A000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Selenium automation tests for register feature
</commit_message>
<xml_diff>
--- a/TestCases/Register_TestCase.xlsx
+++ b/TestCases/Register_TestCase.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DoAnNganh\SpringMediCareWeb-Selenium-Testing\TestCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B75FE8B-1885-45F1-A7A9-8A48D5CA5FF4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60793AD2-8272-4015-8711-01D383C7DACF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -522,7 +522,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="d\-m"/>
+    <numFmt numFmtId="164" formatCode="d\-m"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -784,7 +784,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
@@ -795,32 +795,32 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1062,9 +1062,9 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -1091,9 +1091,9 @@
     </row>
     <row r="2" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -1122,11 +1122,11 @@
       <c r="A3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="23"/>
-      <c r="D3" s="25"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="26"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -1155,11 +1155,11 @@
       <c r="A4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="31" t="s">
+      <c r="B4" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="23"/>
-      <c r="D4" s="25"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="26"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -1188,11 +1188,11 @@
       <c r="A5" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="23"/>
-      <c r="D5" s="25"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="26"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -1222,7 +1222,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="6">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>3</v>
@@ -1259,7 +1259,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>5</v>
@@ -1321,39 +1321,39 @@
       <c r="AA8" s="3"/>
     </row>
     <row r="9" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A9" s="32" t="s">
+      <c r="A9" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="32" t="s">
+      <c r="C9" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="34" t="s">
+      <c r="D9" s="37" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="29"/>
-      <c r="F9" s="29"/>
-      <c r="G9" s="32" t="s">
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="35" t="s">
+      <c r="H9" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="I9" s="35" t="s">
+      <c r="I9" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="J9" s="35" t="s">
+      <c r="J9" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="K9" s="35" t="s">
+      <c r="K9" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="L9" s="35" t="s">
+      <c r="L9" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="M9" s="35" t="s">
+      <c r="M9" s="27" t="s">
         <v>20</v>
       </c>
       <c r="N9" s="3"/>
@@ -1372,19 +1372,19 @@
       <c r="AA9" s="3"/>
     </row>
     <row r="10" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A10" s="24"/>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="24"/>
-      <c r="J10" s="24"/>
-      <c r="K10" s="24"/>
-      <c r="L10" s="24"/>
-      <c r="M10" s="24"/>
+      <c r="A10" s="28"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="28"/>
+      <c r="D10" s="38"/>
+      <c r="E10" s="33"/>
+      <c r="F10" s="33"/>
+      <c r="G10" s="28"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="28"/>
+      <c r="J10" s="28"/>
+      <c r="K10" s="28"/>
+      <c r="L10" s="28"/>
+      <c r="M10" s="28"/>
       <c r="N10" s="3"/>
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
@@ -1406,14 +1406,14 @@
       <c r="C11" s="11"/>
       <c r="D11" s="11"/>
       <c r="E11" s="11"/>
-      <c r="F11" s="36"/>
-      <c r="G11" s="23"/>
-      <c r="H11" s="23"/>
-      <c r="I11" s="23"/>
-      <c r="J11" s="23"/>
-      <c r="K11" s="23"/>
-      <c r="L11" s="23"/>
-      <c r="M11" s="23"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="24"/>
+      <c r="H11" s="24"/>
+      <c r="I11" s="24"/>
+      <c r="J11" s="24"/>
+      <c r="K11" s="24"/>
+      <c r="L11" s="24"/>
+      <c r="M11" s="24"/>
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
@@ -1430,21 +1430,21 @@
       <c r="AA11" s="3"/>
     </row>
     <row r="12" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A12" s="37" t="s">
+      <c r="A12" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="23"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="23"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23"/>
-      <c r="H12" s="23"/>
-      <c r="I12" s="23"/>
-      <c r="J12" s="23"/>
-      <c r="K12" s="23"/>
-      <c r="L12" s="23"/>
-      <c r="M12" s="25"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="24"/>
+      <c r="I12" s="24"/>
+      <c r="J12" s="24"/>
+      <c r="K12" s="24"/>
+      <c r="L12" s="24"/>
+      <c r="M12" s="26"/>
       <c r="N12" s="3"/>
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
@@ -1470,11 +1470,11 @@
       <c r="C13" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="38" t="s">
+      <c r="D13" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="23"/>
-      <c r="F13" s="23"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="24"/>
       <c r="G13" s="17" t="s">
         <v>30</v>
       </c>
@@ -1506,21 +1506,21 @@
       <c r="AA13" s="3"/>
     </row>
     <row r="14" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A14" s="37" t="s">
+      <c r="A14" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="23"/>
-      <c r="C14" s="23"/>
-      <c r="D14" s="23"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23"/>
-      <c r="H14" s="23"/>
-      <c r="I14" s="23"/>
-      <c r="J14" s="23"/>
-      <c r="K14" s="23"/>
-      <c r="L14" s="23"/>
-      <c r="M14" s="25"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="24"/>
+      <c r="I14" s="24"/>
+      <c r="J14" s="24"/>
+      <c r="K14" s="24"/>
+      <c r="L14" s="24"/>
+      <c r="M14" s="26"/>
       <c r="N14" s="3"/>
       <c r="O14" s="3"/>
       <c r="P14" s="3"/>
@@ -1546,11 +1546,11 @@
       <c r="C15" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="D15" s="38" t="s">
+      <c r="D15" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="E15" s="23"/>
-      <c r="F15" s="23"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="24"/>
       <c r="G15" s="17" t="s">
         <v>36</v>
       </c>
@@ -1591,11 +1591,11 @@
       <c r="C16" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="D16" s="38" t="s">
+      <c r="D16" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
       <c r="G16" s="17" t="s">
         <v>42</v>
       </c>
@@ -1636,11 +1636,11 @@
       <c r="C17" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="D17" s="38" t="s">
+      <c r="D17" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="23"/>
-      <c r="F17" s="23"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
       <c r="G17" s="17" t="s">
         <v>47</v>
       </c>
@@ -1681,11 +1681,11 @@
       <c r="C18" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="D18" s="38" t="s">
+      <c r="D18" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="E18" s="23"/>
-      <c r="F18" s="23"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
       <c r="G18" s="17" t="s">
         <v>52</v>
       </c>
@@ -1726,11 +1726,11 @@
       <c r="C19" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="D19" s="38" t="s">
+      <c r="D19" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="E19" s="23"/>
-      <c r="F19" s="23"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24"/>
       <c r="G19" s="17" t="s">
         <v>57</v>
       </c>
@@ -1771,11 +1771,11 @@
       <c r="C20" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="D20" s="38" t="s">
+      <c r="D20" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="E20" s="23"/>
-      <c r="F20" s="23"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
       <c r="G20" s="17" t="s">
         <v>61</v>
       </c>
@@ -1816,11 +1816,11 @@
       <c r="C21" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="D21" s="38" t="s">
+      <c r="D21" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="E21" s="23"/>
-      <c r="F21" s="23"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
       <c r="G21" s="17" t="s">
         <v>65</v>
       </c>
@@ -1861,11 +1861,11 @@
       <c r="C22" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="D22" s="38" t="s">
+      <c r="D22" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="E22" s="23"/>
-      <c r="F22" s="23"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
       <c r="G22" s="17" t="s">
         <v>70</v>
       </c>
@@ -1897,21 +1897,21 @@
       <c r="AA22" s="3"/>
     </row>
     <row r="23" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A23" s="37" t="s">
+      <c r="A23" s="25" t="s">
         <v>71</v>
       </c>
-      <c r="B23" s="23"/>
-      <c r="C23" s="23"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="23"/>
-      <c r="G23" s="23"/>
-      <c r="H23" s="23"/>
-      <c r="I23" s="23"/>
-      <c r="J23" s="23"/>
-      <c r="K23" s="23"/>
-      <c r="L23" s="23"/>
-      <c r="M23" s="25"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="24"/>
+      <c r="I23" s="24"/>
+      <c r="J23" s="24"/>
+      <c r="K23" s="24"/>
+      <c r="L23" s="24"/>
+      <c r="M23" s="26"/>
       <c r="N23" s="3"/>
       <c r="O23" s="3"/>
       <c r="P23" s="3"/>
@@ -1937,11 +1937,11 @@
       <c r="C24" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="D24" s="38" t="s">
+      <c r="D24" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="E24" s="23"/>
-      <c r="F24" s="23"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="24"/>
       <c r="G24" s="17" t="s">
         <v>76</v>
       </c>
@@ -1982,11 +1982,11 @@
       <c r="C25" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="D25" s="38" t="s">
+      <c r="D25" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="E25" s="23"/>
-      <c r="F25" s="23"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="24"/>
       <c r="G25" s="17" t="s">
         <v>82</v>
       </c>
@@ -2033,11 +2033,11 @@
       <c r="C26" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="D26" s="38" t="s">
+      <c r="D26" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="E26" s="23"/>
-      <c r="F26" s="23"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
       <c r="G26" s="17" t="s">
         <v>89</v>
       </c>
@@ -2078,11 +2078,11 @@
       <c r="C27" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="D27" s="38" t="s">
+      <c r="D27" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="E27" s="23"/>
-      <c r="F27" s="23"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="24"/>
       <c r="G27" s="17" t="s">
         <v>95</v>
       </c>
@@ -2129,11 +2129,11 @@
       <c r="C28" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="D28" s="38" t="s">
+      <c r="D28" s="23" t="s">
         <v>101</v>
       </c>
-      <c r="E28" s="23"/>
-      <c r="F28" s="23"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
       <c r="G28" s="17" t="s">
         <v>102</v>
       </c>
@@ -2180,11 +2180,11 @@
       <c r="C29" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="D29" s="38" t="s">
+      <c r="D29" s="23" t="s">
         <v>108</v>
       </c>
-      <c r="E29" s="23"/>
-      <c r="F29" s="23"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="24"/>
       <c r="G29" s="17" t="s">
         <v>109</v>
       </c>
@@ -2231,11 +2231,11 @@
       <c r="C30" s="16" t="s">
         <v>114</v>
       </c>
-      <c r="D30" s="38" t="s">
+      <c r="D30" s="23" t="s">
         <v>115</v>
       </c>
-      <c r="E30" s="23"/>
-      <c r="F30" s="23"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="24"/>
       <c r="G30" s="17" t="s">
         <v>116</v>
       </c>
@@ -2282,11 +2282,11 @@
       <c r="C31" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="D31" s="38" t="s">
+      <c r="D31" s="23" t="s">
         <v>122</v>
       </c>
-      <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="24"/>
       <c r="G31" s="17" t="s">
         <v>123</v>
       </c>
@@ -2324,21 +2324,21 @@
       <c r="AA31" s="3"/>
     </row>
     <row r="32" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A32" s="37" t="s">
+      <c r="A32" s="25" t="s">
         <v>126</v>
       </c>
-      <c r="B32" s="23"/>
-      <c r="C32" s="23"/>
-      <c r="D32" s="23"/>
-      <c r="E32" s="23"/>
-      <c r="F32" s="23"/>
-      <c r="G32" s="23"/>
-      <c r="H32" s="23"/>
-      <c r="I32" s="23"/>
-      <c r="J32" s="23"/>
-      <c r="K32" s="23"/>
-      <c r="L32" s="23"/>
-      <c r="M32" s="25"/>
+      <c r="B32" s="24"/>
+      <c r="C32" s="24"/>
+      <c r="D32" s="24"/>
+      <c r="E32" s="24"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="24"/>
+      <c r="I32" s="24"/>
+      <c r="J32" s="24"/>
+      <c r="K32" s="24"/>
+      <c r="L32" s="24"/>
+      <c r="M32" s="26"/>
       <c r="N32" s="3"/>
       <c r="O32" s="3"/>
       <c r="P32" s="3"/>
@@ -2364,11 +2364,11 @@
       <c r="C33" s="16" t="s">
         <v>129</v>
       </c>
-      <c r="D33" s="38" t="s">
+      <c r="D33" s="23" t="s">
         <v>130</v>
       </c>
-      <c r="E33" s="23"/>
-      <c r="F33" s="23"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="24"/>
       <c r="G33" s="17" t="s">
         <v>131</v>
       </c>
@@ -2415,11 +2415,11 @@
       <c r="C34" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="D34" s="38" t="s">
+      <c r="D34" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="E34" s="23"/>
-      <c r="F34" s="23"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="24"/>
       <c r="G34" s="17" t="s">
         <v>138</v>
       </c>
@@ -30777,6 +30777,34 @@
     </row>
   </sheetData>
   <mergeCells count="39">
+    <mergeCell ref="B1:D2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:F10"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="M9:M10"/>
+    <mergeCell ref="F11:M11"/>
+    <mergeCell ref="A12:M12"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="A14:M14"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="A23:M23"/>
     <mergeCell ref="D31:F31"/>
     <mergeCell ref="A32:M32"/>
     <mergeCell ref="D33:F33"/>
@@ -30788,34 +30816,6 @@
     <mergeCell ref="D28:F28"/>
     <mergeCell ref="D29:F29"/>
     <mergeCell ref="D30:F30"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="D21:F21"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="A23:M23"/>
-    <mergeCell ref="A14:M14"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="M9:M10"/>
-    <mergeCell ref="F11:M11"/>
-    <mergeCell ref="A12:M12"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="B1:D2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:F10"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="G13" r:id="rId1" xr:uid="{00000000-0004-0000-0300-000000000000}"/>

</xml_diff>

<commit_message>
Refactor register Selenium tests and reporting
</commit_message>
<xml_diff>
--- a/TestCases/Register_TestCase.xlsx
+++ b/TestCases/Register_TestCase.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DoAnNganh\SpringMediCareWeb-Selenium-Testing\TestCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60793AD2-8272-4015-8711-01D383C7DACF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{470389A8-C7CF-43CF-AF63-B97228989C1B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Register" sheetId="4" r:id="rId1"/>
+    <sheet name="REGISTER" sheetId="5" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="ACTION">#REF!</definedName>
@@ -28,16 +28,25 @@
     <t>TEST CASE</t>
   </si>
   <si>
+    <t>System Name：</t>
+  </si>
+  <si>
+    <t>SpringMediCareWeb</t>
+  </si>
+  <si>
+    <t>Module Code：</t>
+  </si>
+  <si>
     <t>Test requirement:</t>
   </si>
   <si>
     <t>Pass</t>
   </si>
   <si>
-    <t>Pending</t>
+    <t>Fail</t>
   </si>
   <si>
-    <t>Fail</t>
+    <t>Pending</t>
   </si>
   <si>
     <t>Number of test cases:</t>
@@ -67,18 +76,6 @@
     <t>Note</t>
   </si>
   <si>
-    <t>System Name：</t>
-  </si>
-  <si>
-    <t>SpringMediCareWeb</t>
-  </si>
-  <si>
-    <t>Module Code：</t>
-  </si>
-  <si>
-    <t>AUTH100 - Authentication</t>
-  </si>
-  <si>
     <t>Retest Date</t>
   </si>
   <si>
@@ -94,30 +91,23 @@
     <t>2. Kiểm tra validation dữ liệu bắt buộc</t>
   </si>
   <si>
-    <t>Bỏ trống tên đăng nhập</t>
+    <t>AUTH - Register</t>
   </si>
   <si>
-    <t>Bỏ trống mật khẩu</t>
-  </si>
-  <si>
-    <t>AUTH1 - Register</t>
+    <t>User Registration</t>
   </si>
   <si>
     <t>TC-REGISTER-001</t>
   </si>
   <si>
-    <t>Đăng ký thành công với thông tin hợp lệ</t>
+    <t>Kiểm tra đăng ký tài khoản với thông tin hợp lệ</t>
   </si>
   <si>
-    <t>1: Mở trang đăng ký.
-2: Nhập họ và tên hợp lệ.
-3: Nhập email chưa tồn tại.
-4: Nhập số điện thoại hợp lệ.
-5: Nhập tên đăng nhập chưa tồn tại.
-6: Nhập mật khẩu hợp lệ.
-7: Nhập xác nhận mật khẩu trùng khớp.
-8: Chọn ảnh đại diện hợp lệ.
-9: Nhấn nút Đăng ký.</t>
+    <t>1: Mở trang đăng ký. 
+2: Nhập đầy đủ thông tin hợp lệ. 
+3: Chọn ảnh đại diện hợp lệ. 
+4: Nhấn nút Đăng ký. 
+5: Kiểm tra kết quả sau khi nhấn Đăng ký.</t>
   </si>
   <si>
     <t>Hệ thống tạo tài khoản thành công, hiển thị thông báo phù hợp và chuyển người dùng đến trang đăng nhập.</t>
@@ -132,13 +122,14 @@
     <t>TC-REGISTER-002</t>
   </si>
   <si>
-    <t>Đăng ký khi không chọn ảnh đại diện</t>
+    <t>Kiểm tra đăng ký khi không chọn ảnh đại diện</t>
   </si>
   <si>
-    <t>1: Mở trang đăng ký.
-2: Nhập đầy đủ thông tin hợp lệ.
-3: Không chọn ảnh đại diện.
-4: Nhấn nút Đăng ký.</t>
+    <t>1: Mở trang đăng ký. 
+2: Nhập đầy đủ thông tin hợp lệ. 
+3: Không chọn ảnh đại diện. 
+4: Nhấn nút Đăng ký. 
+5: Kiểm tra kết quả sau khi nhấn Đăng ký.</t>
   </si>
   <si>
     <t>Hệ thống không tạo tài khoản và hiển thị thông báo yêu cầu chọn ảnh đại diện.</t>
@@ -153,13 +144,14 @@
     <t>TC-REGISTER-003</t>
   </si>
   <si>
-    <t>Bỏ trống họ</t>
+    <t>Kiểm tra đăng ký khi bỏ trống họ</t>
   </si>
   <si>
-    <t>1: Mở trang đăng ký.
-2: Để trống trường Họ.
-3: Nhập hợp lệ các trường còn lại.
-4: Nhấn nút Đăng ký.</t>
+    <t>1: Mở trang đăng ký. 
+2: Để trống trường Họ. 
+3: Nhập hợp lệ các trường còn lại. 
+4: Nhấn nút Đăng ký. 
+5: Kiểm tra kết quả sau khi nhấn Đăng ký.</t>
   </si>
   <si>
     <t>Hệ thống không tạo tài khoản và hiển thị yêu cầu nhập họ.</t>
@@ -171,13 +163,14 @@
     <t>TC-REGISTER-004</t>
   </si>
   <si>
-    <t>Bỏ trống tên</t>
+    <t>Kiểm tra đăng ký khi bỏ trống tên</t>
   </si>
   <si>
-    <t>1: Mở trang đăng ký.
-2: Để trống trường Tên.
-3: Nhập hợp lệ các trường còn lại.
-4: Nhấn nút Đăng ký.</t>
+    <t>1: Mở trang đăng ký. 
+2: Để trống trường Tên. 
+3: Nhập hợp lệ các trường còn lại. 
+4: Nhấn nút Đăng ký. 
+5: Kiểm tra kết quả sau khi nhấn Đăng ký.</t>
   </si>
   <si>
     <t>Hệ thống không tạo tài khoản và hiển thị yêu cầu nhập tên.</t>
@@ -189,13 +182,14 @@
     <t>TC-REGISTER-005</t>
   </si>
   <si>
-    <t>Bỏ trống email</t>
+    <t>Kiểm tra đăng ký khi bỏ trống email</t>
   </si>
   <si>
-    <t>1: Mở trang đăng ký.
-2: Để trống trường Email.
-3: Nhập hợp lệ các trường còn lại.
-4: Nhấn nút Đăng ký.</t>
+    <t>1: Mở trang đăng ký. 
+2: Để trống trường Email. 
+3: Nhập hợp lệ các trường còn lại. 
+4: Nhấn nút Đăng ký. 
+5: Kiểm tra kết quả sau khi nhấn Đăng ký.</t>
   </si>
   <si>
     <t>Hệ thống không tạo tài khoản và hiển thị yêu cầu nhập email.</t>
@@ -207,13 +201,14 @@
     <t>TC-REGISTER-006</t>
   </si>
   <si>
-    <t>Bỏ trống số điện thoại</t>
+    <t>Kiểm tra đăng ký khi bỏ trống số điện thoại</t>
   </si>
   <si>
-    <t>1: Mở trang đăng ký.
-2: Để trống trường Số điện thoại.
-3: Nhập hợp lệ các trường còn lại.
-4: Nhấn nút Đăng ký.</t>
+    <t>1: Mở trang đăng ký. 
+2: Để trống trường Số điện thoại. 
+3: Nhập hợp lệ các trường còn lại. 
+4: Nhấn nút Đăng ký. 
+5: Kiểm tra kết quả sau khi nhấn Đăng ký.</t>
   </si>
   <si>
     <t>Hệ thống không tạo tài khoản và hiển thị yêu cầu nhập số điện thoại.</t>
@@ -225,10 +220,14 @@
     <t>TC-REGISTER-007</t>
   </si>
   <si>
-    <t>1: Mở trang đăng ký.
-2: Để trống trường Tên đăng nhập.
-3: Nhập hợp lệ các trường còn lại.
-4: Nhấn nút Đăng ký.</t>
+    <t>Kiểm tra đăng ký khi bỏ trống tên đăng nhập</t>
+  </si>
+  <si>
+    <t>1: Mở trang đăng ký. 
+2: Để trống trường Tên đăng nhập. 
+3: Nhập hợp lệ các trường còn lại. 
+4: Nhấn nút Đăng ký. 
+5: Kiểm tra kết quả sau khi nhấn Đăng ký.</t>
   </si>
   <si>
     <t>Hệ thống không tạo tài khoản và hiển thị yêu cầu nhập tên đăng nhập.</t>
@@ -240,10 +239,14 @@
     <t>TC-REGISTER-008</t>
   </si>
   <si>
-    <t>1: Mở trang đăng ký.
-2: Để trống trường Mật khẩu.
-3: Nhập hợp lệ các trường còn lại.
-4: Nhấn nút Đăng ký.</t>
+    <t>Kiểm tra đăng ký khi bỏ trống mật khẩu</t>
+  </si>
+  <si>
+    <t>1: Mở trang đăng ký. 
+2: Để trống trường Mật khẩu. 
+3: Nhập hợp lệ các trường còn lại. 
+4: Nhấn nút Đăng ký. 
+5: Kiểm tra kết quả sau khi nhấn Đăng ký.</t>
   </si>
   <si>
     <t>Hệ thống không tạo tài khoản và hiển thị yêu cầu nhập mật khẩu.</t>
@@ -255,13 +258,14 @@
     <t>TC-REGISTER-009</t>
   </si>
   <si>
-    <t>Bỏ trống xác nhận mật khẩu</t>
+    <t>Kiểm tra đăng ký khi bỏ trống xác nhận mật khẩu</t>
   </si>
   <si>
-    <t>1: Mở trang đăng ký.
-2: Để trống trường Xác nhận mật khẩu.
-3: Nhập hợp lệ các trường còn lại.
-4: Nhấn nút Đăng ký.</t>
+    <t>1: Mở trang đăng ký. 
+2: Để trống trường Xác nhận mật khẩu. 
+3: Nhập hợp lệ các trường còn lại. 
+4: Nhấn nút Đăng ký. 
+5: Kiểm tra kết quả sau khi nhấn Đăng ký.</t>
   </si>
   <si>
     <t>Hệ thống không tạo tài khoản và hiển thị yêu cầu nhập xác nhận mật khẩu.</t>
@@ -276,13 +280,14 @@
     <t>TC-REGISTER-010</t>
   </si>
   <si>
-    <t>Đăng ký với email không đúng định dạng</t>
+    <t>Kiểm tra đăng ký với email sai định dạng</t>
   </si>
   <si>
-    <t>1: Mở trang đăng ký.
-2: Nhập email không đúng định dạng, ví dụ kimphunggmail.com.
-3: Nhập hợp lệ các trường còn lại.
-4: Nhấn nút Đăng ký.</t>
+    <t>1: Mở trang đăng ký. 
+2: Nhập email sai định dạng. 
+3: Nhập hợp lệ các trường còn lại. 
+4: Nhấn nút Đăng ký. 
+5: Kiểm tra kết quả sau khi nhấn Đăng ký.</t>
   </si>
   <si>
     <t>Hệ thống không tạo tài khoản và hiển thị thông báo email không hợp lệ.</t>
@@ -297,13 +302,14 @@
     <t>TC-REGISTER-011</t>
   </si>
   <si>
-    <t>Đăng ký với số điện thoại không đúng định dạng</t>
+    <t>Kiểm tra đăng ký với số điện thoại sai định dạng</t>
   </si>
   <si>
-    <t>1: Mở trang đăng ký.
-2: Nhập số điện thoại gồm 11 chữ số.
-3: Nhập hợp lệ các trường còn lại.
-4: Nhấn nút Đăng ký.</t>
+    <t>1: Mở trang đăng ký. 
+2: Nhập số điện thoại 11 chữ số. 
+3: Nhập hợp lệ các trường còn lại. 
+4: Nhấn nút Đăng ký. 
+5: Kiểm tra kết quả sau khi nhấn Đăng ký.</t>
   </si>
   <si>
     <t>Hệ thống không tạo tài khoản và hiển thị thông báo số điện thoại không hợp lệ.</t>
@@ -321,14 +327,14 @@
     <t>TC-REGISTER-012</t>
   </si>
   <si>
-    <t>Xác nhận mật khẩu không khớp</t>
+    <t>Kiểm tra đăng ký khi xác nhận mật khẩu không khớp</t>
   </si>
   <si>
-    <t>1: Mở trang đăng ký.
-2: Nhập mật khẩu hợp lệ.
-3: Nhập xác nhận mật khẩu khác với mật khẩu đã nhập.
-4: Nhập hợp lệ các trường còn lại.
-5: Nhấn nút Đăng ký.</t>
+    <t>1: Mở trang đăng ký. 
+2: Nhập mật khẩu hợp lệ và xác nhận mật khẩu không khớp. 
+3: Nhập hợp lệ các trường còn lại. 
+4: Nhấn nút Đăng ký. 
+5: Kiểm tra kết quả sau khi nhấn Đăng ký.</t>
   </si>
   <si>
     <t>Hệ thống không tạo tài khoản và hiển thị thông báo xác nhận mật khẩu không khớp.</t>
@@ -343,14 +349,15 @@
     <t>TC-REGISTER-013</t>
   </si>
   <si>
-    <t>Đăng ký với mật khẩu ngắn hơn 7 ký tự</t>
+    <t>Kiểm tra đăng ký với mật khẩu ngắn hơn 7 ký tự</t>
   </si>
   <si>
     <t>1: Mở trang đăng ký.
 2: Nhập mật khẩu ngắn hơn 7 ký tự 
 3: Nhập xác nhận mật khẩu trùng khớp.
 4: Nhập hợp lệ các trường còn lại.
-5: Nhấn nút Đăng ký.</t>
+5: Nhấn nút Đăng ký.
+6: Kiểm tra kết quả sau khi nhấn Đăng ký.</t>
   </si>
   <si>
     <t>Hệ thống không tạo tài khoản và hiển thị thông báo mật khẩu không hợp lệ.</t>
@@ -368,14 +375,15 @@
     <t>TC-REGISTER-014</t>
   </si>
   <si>
-    <t>Đăng ký với mật khẩu không chứa chữ in hoa</t>
+    <t>Kiểm tra đăng ký với mật khẩu không có chữ in hoa</t>
   </si>
   <si>
     <t>1: Mở trang đăng ký.
 2: Nhập mật khẩu không có chữ in hoa, có số, có chữ thường và ký tự đặc biệt 
 3: Nhập xác nhận mật khẩu trùng khớp.
 4: Nhập hợp lệ các trường còn lại.
-5: Nhấn nút Đăng ký.</t>
+5: Nhấn nút Đăng ký.
+6: Kiểm tra kết quả sau khi nhấn Đăng ký.</t>
   </si>
   <si>
     <t>Hệ thống không tạo tài khoản và hiển thị thông báo mật khẩu phải chứa ít nhất một chữ in hoa.</t>
@@ -393,14 +401,15 @@
     <t>TC-REGISTER-015</t>
   </si>
   <si>
-    <t>Đăng ký với mật khẩu không chứa chữ thường</t>
+    <t>Kiểm tra đăng ký với mật khẩu không có chữ thường</t>
   </si>
   <si>
     <t>1: Mở trang đăng ký.
 2: Nhập mật khẩu không có chữ thường, có số, có chữ hoa và ký tự đặc biệt 
 3: Nhập xác nhận mật khẩu trùng khớp.
 4: Nhập hợp lệ các trường còn lại.
-5: Nhấn nút Đăng ký.</t>
+5: Nhấn nút Đăng ký.
+6: Kiểm tra kết quả sau khi nhấn Đăng ký.</t>
   </si>
   <si>
     <t>Hệ thống không tạo tài khoản và hiển thị thông báo mật khẩu phải chứa ít nhất một chữ thường.</t>
@@ -418,14 +427,15 @@
     <t>TC-REGISTER-016</t>
   </si>
   <si>
-    <t>Đăng ký với mật khẩu không chứa số</t>
+    <t>Kiểm tra đăng ký với mật khẩu không có chữ số</t>
   </si>
   <si>
     <t>1: Mở trang đăng ký.
 2: Nhập mật khẩu không có số, có chữ thường, có chữ hoa và ký tự đặc biệt 
 3: Nhập xác nhận mật khẩu trùng khớp.
 4: Nhập hợp lệ các trường còn lại.
-5: Nhấn nút Đăng ký.</t>
+5: Nhấn nút Đăng ký.
+6: Kiểm tra kết quả sau khi nhấn Đăng ký.</t>
   </si>
   <si>
     <t>Hệ thống không tạo tài khoản và hiển thị thông báo mật khẩu phải chứa ít nhất một chữ số.</t>
@@ -443,14 +453,15 @@
     <t>TC-REGISTER-017</t>
   </si>
   <si>
-    <t xml:space="preserve">Đăng ký với mật khẩu không chứa ký tự đặc biệt </t>
+    <t>Kiểm tra đăng ký với mật khẩu không có ký tự đặc biệt</t>
   </si>
   <si>
     <t>1: Mở trang đăng ký.
 2: Nhập mật khẩu không có ký tự đặc biệt, có số, có chữ thường, có chữ hoa  
 3: Nhập xác nhận mật khẩu trùng khớp.
 4: Nhập hợp lệ các trường còn lại.
-5: Nhấn nút Đăng ký.</t>
+5: Nhấn nút Đăng ký.
+6: Kiểm tra kết quả sau khi nhấn Đăng ký.</t>
   </si>
   <si>
     <t>Hệ thống không tạo tài khoản và hiển thị thông báo mật khẩu phải chứa ít nhất một ký tự đặc biệt.</t>
@@ -471,13 +482,14 @@
     <t>TC-REGISTER-018</t>
   </si>
   <si>
-    <t>Đăng ký với tên đăng nhập đã tồn tại</t>
+    <t>Kiểm tra đăng ký với tên đăng nhập đã tồn tại</t>
   </si>
   <si>
     <t>1: Mở trang đăng ký.
 2: Nhập tên đăng nhập là patient_an đã có trong hệ thống.
 3: Nhập hợp lệ các trường còn lại.
-4: Nhấn nút Đăng ký.</t>
+4: Nhấn nút Đăng ký.
+5: Kiểm tra kết quả sau khi nhấn Đăng ký.</t>
   </si>
   <si>
     <t xml:space="preserve">Hệ thống không tạo tài khoản và hiển thị thông báo tên đăng nhập đã tồn tại.
@@ -496,13 +508,14 @@
     <t>TC-REGISTER-019</t>
   </si>
   <si>
-    <t>Đăng ký với email đã tồn tại</t>
+    <t>Kiểm tra đăng ký với email đã tồn tại</t>
   </si>
   <si>
     <t>1: Mở trang đăng ký.
 2: Nhập email là an@gmail.com đã có trong hệ thống.
 3: Nhập hợp lệ các trường còn lại.
-4: Nhấn nút Đăng ký.</t>
+4: Nhấn nút Đăng ký.
+5: Kiểm tra kết quả sau khi nhấn Đăng ký.</t>
   </si>
   <si>
     <t>Hệ thống không tạo tài khoản và hiển thị thông báo email đã tồn tại.</t>
@@ -522,7 +535,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="d\-m"/>
+    <numFmt numFmtId="165" formatCode="d\-m"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -537,10 +550,6 @@
       <name val="Tahoma"/>
     </font>
     <font>
-      <sz val="11"/>
-      <name val="MS PGothic"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
@@ -550,6 +559,10 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="MS PGothic"/>
     </font>
     <font>
       <b/>
@@ -626,6 +639,30 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
@@ -650,9 +687,7 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
+      <left/>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
@@ -662,6 +697,26 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -701,126 +756,81 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="38">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1039,7 +1049,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -1062,9 +1072,9 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -1091,9 +1101,9 @@
     </row>
     <row r="2" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -1120,13 +1130,13 @@
     </row>
     <row r="3" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>14</v>
+        <v>1</v>
       </c>
-      <c r="B3" s="34" t="s">
-        <v>15</v>
+      <c r="B3" s="26" t="s">
+        <v>2</v>
       </c>
-      <c r="C3" s="24"/>
-      <c r="D3" s="26"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="28"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -1153,13 +1163,13 @@
     </row>
     <row r="4" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>16</v>
+        <v>3</v>
       </c>
-      <c r="B4" s="35" t="s">
-        <v>17</v>
+      <c r="B4" s="26" t="s">
+        <v>22</v>
       </c>
-      <c r="C4" s="24"/>
-      <c r="D4" s="26"/>
+      <c r="C4" s="27"/>
+      <c r="D4" s="28"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -1186,13 +1196,13 @@
     </row>
     <row r="5" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
-      <c r="B5" s="34" t="s">
-        <v>25</v>
+      <c r="B5" s="26" t="s">
+        <v>23</v>
       </c>
-      <c r="C5" s="24"/>
-      <c r="D5" s="26"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="28"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -1219,13 +1229,13 @@
     </row>
     <row r="6" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B6" s="6">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D6" s="8">
         <v>0</v>
@@ -1256,13 +1266,13 @@
     </row>
     <row r="7" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B7" s="6">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D7" s="8">
         <v>19</v>
@@ -1321,40 +1331,40 @@
       <c r="AA8" s="3"/>
     </row>
     <row r="9" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A9" s="30" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="36" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9" s="30" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" s="37" t="s">
+      <c r="A9" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="32"/>
-      <c r="F9" s="32"/>
-      <c r="G9" s="30" t="s">
+      <c r="B9" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="27" t="s">
+      <c r="C9" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="I9" s="27" t="s">
+      <c r="D9" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="J9" s="27" t="s">
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="K9" s="27" t="s">
+      <c r="H9" s="34" t="s">
+        <v>14</v>
+      </c>
+      <c r="I9" s="34" t="s">
+        <v>15</v>
+      </c>
+      <c r="J9" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="K9" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="L9" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="L9" s="27" t="s">
+      <c r="M9" s="34" t="s">
         <v>19</v>
-      </c>
-      <c r="M9" s="27" t="s">
-        <v>20</v>
       </c>
       <c r="N9" s="3"/>
       <c r="O9" s="3"/>
@@ -1372,19 +1382,19 @@
       <c r="AA9" s="3"/>
     </row>
     <row r="10" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A10" s="28"/>
-      <c r="B10" s="28"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="38"/>
-      <c r="E10" s="33"/>
-      <c r="F10" s="33"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="28"/>
-      <c r="J10" s="28"/>
-      <c r="K10" s="28"/>
-      <c r="L10" s="28"/>
-      <c r="M10" s="28"/>
+      <c r="A10" s="30"/>
+      <c r="B10" s="30"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="33"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="30"/>
+      <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
+      <c r="M10" s="30"/>
       <c r="N10" s="3"/>
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
@@ -1406,14 +1416,14 @@
       <c r="C11" s="11"/>
       <c r="D11" s="11"/>
       <c r="E11" s="11"/>
-      <c r="F11" s="29"/>
-      <c r="G11" s="24"/>
-      <c r="H11" s="24"/>
-      <c r="I11" s="24"/>
-      <c r="J11" s="24"/>
-      <c r="K11" s="24"/>
-      <c r="L11" s="24"/>
-      <c r="M11" s="24"/>
+      <c r="F11" s="35"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="27"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="27"/>
+      <c r="K11" s="27"/>
+      <c r="L11" s="27"/>
+      <c r="M11" s="27"/>
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
@@ -1430,21 +1440,21 @@
       <c r="AA11" s="3"/>
     </row>
     <row r="12" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A12" s="25" t="s">
-        <v>21</v>
+      <c r="A12" s="36" t="s">
+        <v>20</v>
       </c>
-      <c r="B12" s="24"/>
-      <c r="C12" s="24"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="24"/>
-      <c r="F12" s="24"/>
-      <c r="G12" s="24"/>
-      <c r="H12" s="24"/>
-      <c r="I12" s="24"/>
-      <c r="J12" s="24"/>
-      <c r="K12" s="24"/>
-      <c r="L12" s="24"/>
-      <c r="M12" s="26"/>
+      <c r="B12" s="27"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="27"/>
+      <c r="K12" s="27"/>
+      <c r="L12" s="27"/>
+      <c r="M12" s="28"/>
       <c r="N12" s="3"/>
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
@@ -1462,30 +1472,30 @@
     </row>
     <row r="13" spans="1:27" ht="126.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="D13" s="37" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="E13" s="27"/>
+      <c r="F13" s="27"/>
+      <c r="G13" s="17" t="s">
         <v>28</v>
-      </c>
-      <c r="D13" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="E13" s="24"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="17" t="s">
-        <v>30</v>
       </c>
       <c r="H13" s="18">
         <v>46218</v>
       </c>
       <c r="I13" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J13" s="16" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K13" s="19"/>
       <c r="L13" s="3"/>
@@ -1506,21 +1516,21 @@
       <c r="AA13" s="3"/>
     </row>
     <row r="14" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A14" s="25" t="s">
-        <v>22</v>
+      <c r="A14" s="36" t="s">
+        <v>21</v>
       </c>
-      <c r="B14" s="24"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="24"/>
-      <c r="I14" s="24"/>
-      <c r="J14" s="24"/>
-      <c r="K14" s="24"/>
-      <c r="L14" s="24"/>
-      <c r="M14" s="26"/>
+      <c r="B14" s="27"/>
+      <c r="C14" s="27"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="27"/>
+      <c r="I14" s="27"/>
+      <c r="J14" s="27"/>
+      <c r="K14" s="27"/>
+      <c r="L14" s="27"/>
+      <c r="M14" s="28"/>
       <c r="N14" s="3"/>
       <c r="O14" s="3"/>
       <c r="P14" s="3"/>
@@ -1536,32 +1546,32 @@
       <c r="Z14" s="3"/>
       <c r="AA14" s="3"/>
     </row>
-    <row r="15" spans="1:27" ht="69" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:27" ht="82.8" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="15" t="s">
+      <c r="D15" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="17" t="s">
         <v>34</v>
-      </c>
-      <c r="D15" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="E15" s="24"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="17" t="s">
-        <v>36</v>
       </c>
       <c r="H15" s="18">
         <v>46218</v>
       </c>
       <c r="I15" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J15" s="16" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K15" s="18"/>
       <c r="L15" s="14"/>
@@ -1581,32 +1591,32 @@
       <c r="Z15" s="3"/>
       <c r="AA15" s="3"/>
     </row>
-    <row r="16" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" ht="86.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="B16" s="15" t="s">
+      <c r="D16" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="17" t="s">
         <v>40</v>
-      </c>
-      <c r="D16" s="23" t="s">
-        <v>41</v>
-      </c>
-      <c r="E16" s="24"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="17" t="s">
-        <v>42</v>
       </c>
       <c r="H16" s="18">
         <v>46218</v>
       </c>
       <c r="I16" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J16" s="16" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="K16" s="19"/>
       <c r="L16" s="19"/>
@@ -1626,32 +1636,32 @@
       <c r="Z16" s="3"/>
       <c r="AA16" s="3"/>
     </row>
-    <row r="17" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:27" ht="84.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="B17" s="15" t="s">
+      <c r="D17" s="37" t="s">
         <v>44</v>
       </c>
-      <c r="C17" s="16" t="s">
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="17" t="s">
         <v>45</v>
-      </c>
-      <c r="D17" s="23" t="s">
-        <v>46</v>
-      </c>
-      <c r="E17" s="24"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="17" t="s">
-        <v>47</v>
       </c>
       <c r="H17" s="18">
         <v>46218</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J17" s="16" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="K17" s="19"/>
       <c r="L17" s="19"/>
@@ -1671,32 +1681,32 @@
       <c r="Z17" s="3"/>
       <c r="AA17" s="3"/>
     </row>
-    <row r="18" spans="1:27" ht="55.2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:27" ht="82.8" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="C18" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="B18" s="15" t="s">
+      <c r="D18" s="37" t="s">
         <v>49</v>
       </c>
-      <c r="C18" s="16" t="s">
+      <c r="E18" s="27"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="17" t="s">
         <v>50</v>
-      </c>
-      <c r="D18" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="E18" s="24"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="17" t="s">
-        <v>52</v>
       </c>
       <c r="H18" s="18">
         <v>46218</v>
       </c>
       <c r="I18" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J18" s="16" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="K18" s="19"/>
       <c r="L18" s="19"/>
@@ -1716,32 +1726,32 @@
       <c r="Z18" s="3"/>
       <c r="AA18" s="3"/>
     </row>
-    <row r="19" spans="1:27" ht="55.2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:27" ht="82.8" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="B19" s="15" t="s">
+      <c r="D19" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="C19" s="16" t="s">
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="17" t="s">
         <v>55</v>
-      </c>
-      <c r="D19" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="17" t="s">
-        <v>57</v>
       </c>
       <c r="H19" s="18">
         <v>46218</v>
       </c>
       <c r="I19" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J19" s="16" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="K19" s="19"/>
       <c r="L19" s="19"/>
@@ -1761,32 +1771,32 @@
       <c r="Z19" s="3"/>
       <c r="AA19" s="3"/>
     </row>
-    <row r="20" spans="1:27" ht="55.2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:27" ht="82.8" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="C20" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="B20" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="C20" s="16" t="s">
+      <c r="D20" s="37" t="s">
         <v>59</v>
       </c>
-      <c r="D20" s="23" t="s">
+      <c r="E20" s="27"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="17" t="s">
         <v>60</v>
-      </c>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="17" t="s">
-        <v>61</v>
       </c>
       <c r="H20" s="18">
         <v>46218</v>
       </c>
       <c r="I20" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J20" s="16" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K20" s="19"/>
       <c r="L20" s="19"/>
@@ -1806,21 +1816,21 @@
       <c r="Z20" s="3"/>
       <c r="AA20" s="3"/>
     </row>
-    <row r="21" spans="1:27" ht="55.2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:27" ht="82.8" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="C21" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="D21" s="23" t="s">
+      <c r="D21" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
       <c r="G21" s="17" t="s">
         <v>65</v>
       </c>
@@ -1828,7 +1838,7 @@
         <v>46218</v>
       </c>
       <c r="I21" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J21" s="16" t="s">
         <v>64</v>
@@ -1851,7 +1861,7 @@
       <c r="Z21" s="3"/>
       <c r="AA21" s="3"/>
     </row>
-    <row r="22" spans="1:27" ht="55.2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:27" ht="82.8" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
         <v>66</v>
       </c>
@@ -1861,11 +1871,11 @@
       <c r="C22" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="D22" s="23" t="s">
+      <c r="D22" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="E22" s="24"/>
-      <c r="F22" s="24"/>
+      <c r="E22" s="27"/>
+      <c r="F22" s="27"/>
       <c r="G22" s="17" t="s">
         <v>70</v>
       </c>
@@ -1873,7 +1883,7 @@
         <v>46218</v>
       </c>
       <c r="I22" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J22" s="16" t="s">
         <v>69</v>
@@ -1897,21 +1907,21 @@
       <c r="AA22" s="3"/>
     </row>
     <row r="23" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A23" s="25" t="s">
+      <c r="A23" s="36" t="s">
         <v>71</v>
       </c>
-      <c r="B23" s="24"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="24"/>
-      <c r="G23" s="24"/>
-      <c r="H23" s="24"/>
-      <c r="I23" s="24"/>
-      <c r="J23" s="24"/>
-      <c r="K23" s="24"/>
-      <c r="L23" s="24"/>
-      <c r="M23" s="26"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="27"/>
+      <c r="H23" s="27"/>
+      <c r="I23" s="27"/>
+      <c r="J23" s="27"/>
+      <c r="K23" s="27"/>
+      <c r="L23" s="27"/>
+      <c r="M23" s="28"/>
       <c r="N23" s="3"/>
       <c r="O23" s="3"/>
       <c r="P23" s="3"/>
@@ -1937,11 +1947,11 @@
       <c r="C24" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="D24" s="23" t="s">
+      <c r="D24" s="37" t="s">
         <v>75</v>
       </c>
-      <c r="E24" s="24"/>
-      <c r="F24" s="24"/>
+      <c r="E24" s="27"/>
+      <c r="F24" s="27"/>
       <c r="G24" s="17" t="s">
         <v>76</v>
       </c>
@@ -1949,7 +1959,7 @@
         <v>46218</v>
       </c>
       <c r="I24" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J24" s="16" t="s">
         <v>77</v>
@@ -1972,7 +1982,7 @@
       <c r="Z24" s="3"/>
       <c r="AA24" s="3"/>
     </row>
-    <row r="25" spans="1:27" ht="84.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:27" ht="93.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
         <v>78</v>
       </c>
@@ -1982,11 +1992,11 @@
       <c r="C25" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="D25" s="23" t="s">
+      <c r="D25" s="37" t="s">
         <v>81</v>
       </c>
-      <c r="E25" s="24"/>
-      <c r="F25" s="24"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="27"/>
       <c r="G25" s="17" t="s">
         <v>82</v>
       </c>
@@ -1994,7 +2004,7 @@
         <v>46218</v>
       </c>
       <c r="I25" s="14" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J25" s="16" t="s">
         <v>83</v>
@@ -2003,7 +2013,7 @@
         <v>46219</v>
       </c>
       <c r="L25" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M25" s="21" t="s">
         <v>84</v>
@@ -2023,7 +2033,7 @@
       <c r="Z25" s="3"/>
       <c r="AA25" s="3"/>
     </row>
-    <row r="26" spans="1:27" ht="84.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:27" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
         <v>85</v>
       </c>
@@ -2033,11 +2043,11 @@
       <c r="C26" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="D26" s="23" t="s">
+      <c r="D26" s="37" t="s">
         <v>88</v>
       </c>
-      <c r="E26" s="24"/>
-      <c r="F26" s="24"/>
+      <c r="E26" s="27"/>
+      <c r="F26" s="27"/>
       <c r="G26" s="17" t="s">
         <v>89</v>
       </c>
@@ -2045,7 +2055,7 @@
         <v>46218</v>
       </c>
       <c r="I26" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J26" s="16" t="s">
         <v>90</v>
@@ -2078,11 +2088,11 @@
       <c r="C27" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="D27" s="23" t="s">
+      <c r="D27" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="E27" s="24"/>
-      <c r="F27" s="24"/>
+      <c r="E27" s="27"/>
+      <c r="F27" s="27"/>
       <c r="G27" s="17" t="s">
         <v>95</v>
       </c>
@@ -2090,7 +2100,7 @@
         <v>46218</v>
       </c>
       <c r="I27" s="14" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J27" s="16" t="s">
         <v>96</v>
@@ -2099,7 +2109,7 @@
         <v>46219</v>
       </c>
       <c r="L27" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M27" s="21" t="s">
         <v>97</v>
@@ -2129,11 +2139,11 @@
       <c r="C28" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="D28" s="23" t="s">
+      <c r="D28" s="37" t="s">
         <v>101</v>
       </c>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
+      <c r="E28" s="27"/>
+      <c r="F28" s="27"/>
       <c r="G28" s="17" t="s">
         <v>102</v>
       </c>
@@ -2141,7 +2151,7 @@
         <v>46218</v>
       </c>
       <c r="I28" s="14" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J28" s="16" t="s">
         <v>103</v>
@@ -2150,7 +2160,7 @@
         <v>46219</v>
       </c>
       <c r="L28" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M28" s="21" t="s">
         <v>104</v>
@@ -2180,11 +2190,11 @@
       <c r="C29" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="D29" s="23" t="s">
+      <c r="D29" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="E29" s="24"/>
-      <c r="F29" s="24"/>
+      <c r="E29" s="27"/>
+      <c r="F29" s="27"/>
       <c r="G29" s="17" t="s">
         <v>109</v>
       </c>
@@ -2192,7 +2202,7 @@
         <v>46218</v>
       </c>
       <c r="I29" s="14" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J29" s="16" t="s">
         <v>110</v>
@@ -2201,7 +2211,7 @@
         <v>46219</v>
       </c>
       <c r="L29" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M29" s="21" t="s">
         <v>111</v>
@@ -2231,11 +2241,11 @@
       <c r="C30" s="16" t="s">
         <v>114</v>
       </c>
-      <c r="D30" s="23" t="s">
+      <c r="D30" s="37" t="s">
         <v>115</v>
       </c>
-      <c r="E30" s="24"/>
-      <c r="F30" s="24"/>
+      <c r="E30" s="27"/>
+      <c r="F30" s="27"/>
       <c r="G30" s="17" t="s">
         <v>116</v>
       </c>
@@ -2243,7 +2253,7 @@
         <v>46218</v>
       </c>
       <c r="I30" s="14" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J30" s="16" t="s">
         <v>117</v>
@@ -2252,7 +2262,7 @@
         <v>46219</v>
       </c>
       <c r="L30" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M30" s="21" t="s">
         <v>118</v>
@@ -2282,11 +2292,11 @@
       <c r="C31" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="D31" s="23" t="s">
+      <c r="D31" s="37" t="s">
         <v>122</v>
       </c>
-      <c r="E31" s="24"/>
-      <c r="F31" s="24"/>
+      <c r="E31" s="27"/>
+      <c r="F31" s="27"/>
       <c r="G31" s="17" t="s">
         <v>123</v>
       </c>
@@ -2294,7 +2304,7 @@
         <v>46218</v>
       </c>
       <c r="I31" s="14" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J31" s="16" t="s">
         <v>124</v>
@@ -2303,7 +2313,7 @@
         <v>46219</v>
       </c>
       <c r="L31" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M31" s="21" t="s">
         <v>125</v>
@@ -2324,21 +2334,21 @@
       <c r="AA31" s="3"/>
     </row>
     <row r="32" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A32" s="25" t="s">
+      <c r="A32" s="36" t="s">
         <v>126</v>
       </c>
-      <c r="B32" s="24"/>
-      <c r="C32" s="24"/>
-      <c r="D32" s="24"/>
-      <c r="E32" s="24"/>
-      <c r="F32" s="24"/>
-      <c r="G32" s="24"/>
-      <c r="H32" s="24"/>
-      <c r="I32" s="24"/>
-      <c r="J32" s="24"/>
-      <c r="K32" s="24"/>
-      <c r="L32" s="24"/>
-      <c r="M32" s="26"/>
+      <c r="B32" s="27"/>
+      <c r="C32" s="27"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="27"/>
+      <c r="F32" s="27"/>
+      <c r="G32" s="27"/>
+      <c r="H32" s="27"/>
+      <c r="I32" s="27"/>
+      <c r="J32" s="27"/>
+      <c r="K32" s="27"/>
+      <c r="L32" s="27"/>
+      <c r="M32" s="28"/>
       <c r="N32" s="3"/>
       <c r="O32" s="3"/>
       <c r="P32" s="3"/>
@@ -2354,7 +2364,7 @@
       <c r="Z32" s="3"/>
       <c r="AA32" s="3"/>
     </row>
-    <row r="33" spans="1:27" ht="69" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:27" ht="96.6" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
         <v>127</v>
       </c>
@@ -2364,11 +2374,11 @@
       <c r="C33" s="16" t="s">
         <v>129</v>
       </c>
-      <c r="D33" s="23" t="s">
+      <c r="D33" s="37" t="s">
         <v>130</v>
       </c>
-      <c r="E33" s="24"/>
-      <c r="F33" s="24"/>
+      <c r="E33" s="27"/>
+      <c r="F33" s="27"/>
       <c r="G33" s="17" t="s">
         <v>131</v>
       </c>
@@ -2376,7 +2386,7 @@
         <v>46218</v>
       </c>
       <c r="I33" s="14" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J33" s="16" t="s">
         <v>132</v>
@@ -2385,7 +2395,7 @@
         <v>46219</v>
       </c>
       <c r="L33" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M33" s="21" t="s">
         <v>133</v>
@@ -2415,11 +2425,11 @@
       <c r="C34" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="D34" s="23" t="s">
+      <c r="D34" s="37" t="s">
         <v>137</v>
       </c>
-      <c r="E34" s="24"/>
-      <c r="F34" s="24"/>
+      <c r="E34" s="27"/>
+      <c r="F34" s="27"/>
       <c r="G34" s="17" t="s">
         <v>138</v>
       </c>
@@ -2427,7 +2437,7 @@
         <v>46218</v>
       </c>
       <c r="I34" s="14" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J34" s="16" t="s">
         <v>139</v>
@@ -2436,7 +2446,7 @@
         <v>46219</v>
       </c>
       <c r="L34" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M34" s="21" t="s">
         <v>140</v>
@@ -30777,34 +30787,6 @@
     </row>
   </sheetData>
   <mergeCells count="39">
-    <mergeCell ref="B1:D2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:F10"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="M9:M10"/>
-    <mergeCell ref="F11:M11"/>
-    <mergeCell ref="A12:M12"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="A14:M14"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="D21:F21"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="A23:M23"/>
     <mergeCell ref="D31:F31"/>
     <mergeCell ref="A32:M32"/>
     <mergeCell ref="D33:F33"/>
@@ -30816,35 +30798,63 @@
     <mergeCell ref="D28:F28"/>
     <mergeCell ref="D29:F29"/>
     <mergeCell ref="D30:F30"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="A23:M23"/>
+    <mergeCell ref="A14:M14"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="M9:M10"/>
+    <mergeCell ref="F11:M11"/>
+    <mergeCell ref="A12:M12"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="B1:D2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:F10"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="G13" r:id="rId1" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
-    <hyperlink ref="G15" r:id="rId2" xr:uid="{00000000-0004-0000-0300-000001000000}"/>
-    <hyperlink ref="G16" r:id="rId3" xr:uid="{00000000-0004-0000-0300-000002000000}"/>
-    <hyperlink ref="G17" r:id="rId4" xr:uid="{00000000-0004-0000-0300-000003000000}"/>
-    <hyperlink ref="G18" r:id="rId5" xr:uid="{00000000-0004-0000-0300-000004000000}"/>
-    <hyperlink ref="G19" r:id="rId6" xr:uid="{00000000-0004-0000-0300-000005000000}"/>
-    <hyperlink ref="G20" r:id="rId7" xr:uid="{00000000-0004-0000-0300-000006000000}"/>
-    <hyperlink ref="G21" r:id="rId8" xr:uid="{00000000-0004-0000-0300-000007000000}"/>
-    <hyperlink ref="G22" r:id="rId9" xr:uid="{00000000-0004-0000-0300-000008000000}"/>
-    <hyperlink ref="G24" r:id="rId10" xr:uid="{00000000-0004-0000-0300-000009000000}"/>
-    <hyperlink ref="G25" r:id="rId11" xr:uid="{00000000-0004-0000-0300-00000A000000}"/>
-    <hyperlink ref="M25" r:id="rId12" xr:uid="{00000000-0004-0000-0300-00000B000000}"/>
-    <hyperlink ref="G26" r:id="rId13" xr:uid="{00000000-0004-0000-0300-00000C000000}"/>
-    <hyperlink ref="G27" r:id="rId14" xr:uid="{00000000-0004-0000-0300-00000D000000}"/>
-    <hyperlink ref="M27" r:id="rId15" xr:uid="{00000000-0004-0000-0300-00000E000000}"/>
-    <hyperlink ref="G28" r:id="rId16" xr:uid="{00000000-0004-0000-0300-00000F000000}"/>
-    <hyperlink ref="M28" r:id="rId17" xr:uid="{00000000-0004-0000-0300-000010000000}"/>
-    <hyperlink ref="G29" r:id="rId18" xr:uid="{00000000-0004-0000-0300-000011000000}"/>
-    <hyperlink ref="M29" r:id="rId19" xr:uid="{00000000-0004-0000-0300-000012000000}"/>
-    <hyperlink ref="G30" r:id="rId20" xr:uid="{00000000-0004-0000-0300-000013000000}"/>
-    <hyperlink ref="M30" r:id="rId21" xr:uid="{00000000-0004-0000-0300-000014000000}"/>
-    <hyperlink ref="G31" r:id="rId22" xr:uid="{00000000-0004-0000-0300-000015000000}"/>
-    <hyperlink ref="M31" r:id="rId23" xr:uid="{00000000-0004-0000-0300-000016000000}"/>
-    <hyperlink ref="G33" r:id="rId24" xr:uid="{00000000-0004-0000-0300-000017000000}"/>
-    <hyperlink ref="M33" r:id="rId25" xr:uid="{00000000-0004-0000-0300-000018000000}"/>
-    <hyperlink ref="G34" r:id="rId26" xr:uid="{00000000-0004-0000-0300-000019000000}"/>
-    <hyperlink ref="M34" r:id="rId27" xr:uid="{00000000-0004-0000-0300-00001A000000}"/>
+    <hyperlink ref="G13" r:id="rId1" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
+    <hyperlink ref="G15" r:id="rId2" xr:uid="{00000000-0004-0000-0400-000001000000}"/>
+    <hyperlink ref="G16" r:id="rId3" xr:uid="{00000000-0004-0000-0400-000002000000}"/>
+    <hyperlink ref="G17" r:id="rId4" xr:uid="{00000000-0004-0000-0400-000003000000}"/>
+    <hyperlink ref="G18" r:id="rId5" xr:uid="{00000000-0004-0000-0400-000004000000}"/>
+    <hyperlink ref="G19" r:id="rId6" xr:uid="{00000000-0004-0000-0400-000005000000}"/>
+    <hyperlink ref="G20" r:id="rId7" xr:uid="{00000000-0004-0000-0400-000006000000}"/>
+    <hyperlink ref="G21" r:id="rId8" xr:uid="{00000000-0004-0000-0400-000007000000}"/>
+    <hyperlink ref="G22" r:id="rId9" xr:uid="{00000000-0004-0000-0400-000008000000}"/>
+    <hyperlink ref="G24" r:id="rId10" xr:uid="{00000000-0004-0000-0400-000009000000}"/>
+    <hyperlink ref="G25" r:id="rId11" xr:uid="{00000000-0004-0000-0400-00000A000000}"/>
+    <hyperlink ref="M25" r:id="rId12" xr:uid="{00000000-0004-0000-0400-00000B000000}"/>
+    <hyperlink ref="G26" r:id="rId13" xr:uid="{00000000-0004-0000-0400-00000C000000}"/>
+    <hyperlink ref="G27" r:id="rId14" xr:uid="{00000000-0004-0000-0400-00000D000000}"/>
+    <hyperlink ref="M27" r:id="rId15" xr:uid="{00000000-0004-0000-0400-00000E000000}"/>
+    <hyperlink ref="G28" r:id="rId16" xr:uid="{00000000-0004-0000-0400-00000F000000}"/>
+    <hyperlink ref="M28" r:id="rId17" xr:uid="{00000000-0004-0000-0400-000010000000}"/>
+    <hyperlink ref="G29" r:id="rId18" xr:uid="{00000000-0004-0000-0400-000011000000}"/>
+    <hyperlink ref="M29" r:id="rId19" xr:uid="{00000000-0004-0000-0400-000012000000}"/>
+    <hyperlink ref="G30" r:id="rId20" xr:uid="{00000000-0004-0000-0400-000013000000}"/>
+    <hyperlink ref="M30" r:id="rId21" xr:uid="{00000000-0004-0000-0400-000014000000}"/>
+    <hyperlink ref="G31" r:id="rId22" xr:uid="{00000000-0004-0000-0400-000015000000}"/>
+    <hyperlink ref="M31" r:id="rId23" xr:uid="{00000000-0004-0000-0400-000016000000}"/>
+    <hyperlink ref="G33" r:id="rId24" xr:uid="{00000000-0004-0000-0400-000017000000}"/>
+    <hyperlink ref="M33" r:id="rId25" xr:uid="{00000000-0004-0000-0400-000018000000}"/>
+    <hyperlink ref="G34" r:id="rId26" xr:uid="{00000000-0004-0000-0400-000019000000}"/>
+    <hyperlink ref="M34" r:id="rId27" xr:uid="{00000000-0004-0000-0400-00001A000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>